<commit_message>
Route flagged Dev cases to independent adjudication
</commit_message>
<xml_diff>
--- a/workbooks/TurkCuisineBench_Validation_and_Pilot_Workflow_v0.3.xlsx
+++ b/workbooks/TurkCuisineBench_Validation_and_Pilot_Workflow_v0.3.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rdf39e7d1ccdf4f23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dev_Items" sheetId="2" r:id="R6bbb6191f8fc4296"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dev_Reviewer_A" sheetId="3" r:id="Rc1e231015e5a4fd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dev_Reviewer_B" sheetId="4" r:id="R91be41a206314d8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dev_Adjudication" sheetId="5" r:id="R9086a6366b2d4a13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main_Assignment" sheetId="6" r:id="R8927de2c3e974049"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main_Review_Log" sheetId="7" r:id="R9f518aff2f044a09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot_Run_Log" sheetId="8" r:id="R2ae59569844a4cdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="Rddd050bb68b7445f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Reconciliation" sheetId="10" r:id="R216dec7111db4d5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R873e4fda3d724a76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dev_Items" sheetId="2" r:id="Rb0191a1832b74497"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dev_Reviewer_A" sheetId="3" r:id="Red5f3ed3767545fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dev_Reviewer_B" sheetId="4" r:id="Rc045f3eec62d4b9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dev_Adjudication" sheetId="5" r:id="R90b8a3878caf4259"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main_Assignment" sheetId="6" r:id="R78b3ca57cae242ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main_Review_Log" sheetId="7" r:id="Rcd69b21bcfd74c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot_Run_Log" sheetId="8" r:id="R3bc0ccc670ca449f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="9" r:id="R326d42b925d94df7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Reconciliation" sheetId="10" r:id="Rdb2350d2c13c4801"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1027,7 +1027,7 @@
         <x:v>Freeze status</x:v>
       </x:c>
       <x:c r="B30" s="64" t="str">
-        <x:v>NOT FROZEN — pending lead-researcher adjudication</x:v>
+        <x:v>NOT FROZEN — pending independent adjudication</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1080,7 +1080,7 @@
     </x:row>
     <x:row r="2" ht="33" customHeight="1">
       <x:c r="A2" s="45" t="str">
-        <x:v>Raw reviewer forms are archived privately. This sheet is de-identified. Four cases remain pending lead-researcher adjudication; the Dev set is not frozen until those decisions are recorded.</x:v>
+        <x:v>Raw reviewer forms are archived privately. This sheet is de-identified. Four cases remain pending independent adjudication; the Dev set is not frozen until those decisions are recorded.</x:v>
       </x:c>
       <x:c r="B2" s="45"/>
       <x:c r="C2" s="45"/>
@@ -1135,7 +1135,7 @@
         <x:v>issue_type</x:v>
       </x:c>
       <x:c r="M5" s="53" t="str">
-        <x:v>proposed_lead_resolution</x:v>
+        <x:v>author_draft_resolution_not_shown_to_adjudicator</x:v>
       </x:c>
       <x:c r="N5" s="53" t="str">
         <x:v>resolution_status</x:v>
@@ -1232,7 +1232,7 @@
         <x:v>Maraş Tarhanası kurutulurken ürünün serildiği geleneksel hasırın adı nedir?</x:v>
       </x:c>
       <x:c r="N7" s="55" t="str">
-        <x:v>pending_lead_researcher_adjudication</x:v>
+        <x:v>pending_independent_adjudication</x:v>
       </x:c>
       <x:c r="O7" s="55" t="str">
         <x:v>TÜRKPATENT describes çığ as the reed-woven mat on which the tarhana mixture is spread.</x:v>
@@ -2125,7 +2125,7 @@
         <x:v>Afyonkarahisar'da nişan gecesinin ertesi günü oğlan evinin kız evine yaptığı geleneksel yemekli davetin adı nedir?</x:v>
       </x:c>
       <x:c r="N26" s="55" t="str">
-        <x:v>pending_lead_researcher_adjudication</x:v>
+        <x:v>pending_independent_adjudication</x:v>
       </x:c>
       <x:c r="O26" s="55" t="str">
         <x:v>The Ministry of Culture page defines the Zinardı (Sini Ardı) invitation using this event description.</x:v>
@@ -2172,7 +2172,7 @@
         <x:v>Afyonkarahisar sıra yemeklerinde yemeklerin sofraya hangi sırayla getirileceğini düzenleme işine ne ad verilir?</x:v>
       </x:c>
       <x:c r="N27" s="55" t="str">
-        <x:v>pending_lead_researcher_adjudication</x:v>
+        <x:v>pending_independent_adjudication</x:v>
       </x:c>
       <x:c r="O27" s="55" t="str">
         <x:v>The Ministry of Culture page calls arranging the serving order 'Yemek Kurtarma'.</x:v>
@@ -2731,10 +2731,10 @@
         <x:v>missing_required_reviewer_field</x:v>
       </x:c>
       <x:c r="M39" s="55" t="str">
-        <x:v>Accept the item as written after the lead researcher records the missing-field adjudication.</x:v>
+        <x:v>Accept the item as written if the independent adjudicator confirms clarity and source support.</x:v>
       </x:c>
       <x:c r="N39" s="55" t="str">
-        <x:v>pending_lead_researcher_adjudication</x:v>
+        <x:v>pending_independent_adjudication</x:v>
       </x:c>
       <x:c r="O39" s="55" t="str">
         <x:v>The Ministry of Culture page explicitly states that güllaç is associated with Ramadan in Türkiye.</x:v>
@@ -4946,7 +4946,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00110e6cd3d841e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74b604409a534899"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7120,7 +7120,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7f0efa4d6e64c46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48d97f28ae784377"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9296,7 +9296,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8233a9e3c5f5425a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81a0d5f4fb104a04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9496,7 +9496,7 @@
       <x:c r="K7" s="26"/>
       <x:c r="L7" s="26"/>
       <x:c r="M7" s="26" t="str">
-        <x:v>Pending lead-researcher adjudication: concordant_revise_without_proposed_text. Proposed resolution is documented in Review_Reconciliation.</x:v>
+        <x:v>Pending independent adjudication: concordant_revise_without_proposed_text. An author draft is documented in Review_Reconciliation but is not shown in the adjudicator pack.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="46.5" customHeight="1">
@@ -10324,7 +10324,7 @@
       <x:c r="K26" s="26"/>
       <x:c r="L26" s="26"/>
       <x:c r="M26" s="26" t="str">
-        <x:v>Pending lead-researcher adjudication: action_disagreement_and_clarity_concern. Proposed resolution is documented in Review_Reconciliation.</x:v>
+        <x:v>Pending independent adjudication: action_disagreement_and_clarity_concern. An author draft is documented in Review_Reconciliation but is not shown in the adjudicator pack.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="46.5" customHeight="1">
@@ -10360,7 +10360,7 @@
       <x:c r="K27" s="26"/>
       <x:c r="L27" s="26"/>
       <x:c r="M27" s="26" t="str">
-        <x:v>Pending lead-researcher adjudication: field_level_clarity_concern. Proposed resolution is documented in Review_Reconciliation.</x:v>
+        <x:v>Pending independent adjudication: field_level_clarity_concern. An author draft is documented in Review_Reconciliation but is not shown in the adjudicator pack.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="46.5" customHeight="1">
@@ -10880,7 +10880,7 @@
       <x:c r="K39" s="26"/>
       <x:c r="L39" s="26"/>
       <x:c r="M39" s="26" t="str">
-        <x:v>Pending lead-researcher adjudication: missing_required_reviewer_field. Proposed resolution is documented in Review_Reconciliation.</x:v>
+        <x:v>Pending independent adjudication: missing_required_reviewer_field. An author draft is documented in Review_Reconciliation but is not shown in the adjudicator pack.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="46.5" customHeight="1">
@@ -10986,7 +10986,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d9cdc0a325b49de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R539477011e974f9a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17930,7 +17930,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49e23d480f7c4c40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ae2cb43cbdd412c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26114,7 +26114,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7771fa87be7f4f6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c7a9bd0a69a4745"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28633,7 +28633,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7f4d2e04c0445e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c225d5d63a9424b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28732,7 +28732,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="14" t="n">
-        <x:f>COUNTIF('Review_Reconciliation'!$N$6:$N$41,"pending_lead_researcher_adjudication")</x:f>
+        <x:f>COUNTIF('Review_Reconciliation'!$N$6:$N$41,"pending_independent_adjudication")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E6" s="37" t="str">
@@ -28916,7 +28916,7 @@
         <x:v>Interpretation</x:v>
       </x:c>
       <x:c r="B17" s="39" t="str">
-        <x:v>Reviewer evidence has been imported. Four cases require a documented lead-researcher adjudication before the Dev set can be frozen; pilot execution should begin only after that decision and checksum release.</x:v>
+        <x:v>Reviewer evidence has been imported. Four cases require documented independent adjudication before the Dev set can be frozen; pilot execution should begin only after those decisions and the checksum release.</x:v>
       </x:c>
       <x:c r="C17" s="39" t="str"/>
       <x:c r="D17" s="39" t="str"/>

</xml_diff>